<commit_message>
final summary part 1
</commit_message>
<xml_diff>
--- a/summary.xlsx
+++ b/summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\ode-solvers-in-r\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58EC24AF-B08F-4331-88FA-21EC5E537B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4FF0F94-094A-4C9A-B9D9-0EFC48B86819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="58">
   <si>
     <t>Package</t>
   </si>
@@ -51,12 +51,6 @@
     <t>deSolve</t>
   </si>
   <si>
-    <t>ODEPACK + DASPK (FORTRAN)</t>
-  </si>
-  <si>
-    <t>lsoda, lsode, lsodes, lsodar, vode, daspk, radau</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -78,18 +72,9 @@
     <t>DSL</t>
   </si>
   <si>
-    <t>Code-generated C + LSODA-based backend</t>
-  </si>
-  <si>
     <t>mrgsolve</t>
   </si>
   <si>
-    <t>C++ translation of DLSODA</t>
-  </si>
-  <si>
-    <t>lsoda</t>
-  </si>
-  <si>
     <t>Yes (via lsoda)</t>
   </si>
   <si>
@@ -106,9 +91,6 @@
   </si>
   <si>
     <t>Pure R</t>
-  </si>
-  <si>
-    <t>RK4, RK45</t>
   </si>
   <si>
     <t>Νο</t>
@@ -157,12 +139,6 @@
     <t>Simulate dose regimens for pharmacokinetic-pharmacodynamic (PK-PD) models described by differential equation (DE) systems. Simulation using ADVAN-style analytical equations is also supported</t>
   </si>
   <si>
-    <t>Boost::odeint (C++)</t>
-  </si>
-  <si>
-    <t>Adaptive RK (Cash–Karp 5(4)) (RKCK54)</t>
-  </si>
-  <si>
     <t>DAE</t>
   </si>
   <si>
@@ -190,17 +166,47 @@
     <t>Interpreted</t>
   </si>
   <si>
-    <t>Black box solver, cannot change method or solver parameters https://github.com/boostorg/odeint</t>
-  </si>
-  <si>
     <t>DSL(cOde), API-based</t>
+  </si>
+  <si>
+    <t>ode23, ode23s, ode45, ode78</t>
+  </si>
+  <si>
+    <t>Yes (via ode23s)</t>
+  </si>
+  <si>
+    <t>lsoda, lsode, lsodes, lsodar, vode, daspk, bdf, adams, impAdams, radau, euler, rk4, ode23, ode45,  etc.</t>
+  </si>
+  <si>
+    <t>Adaptive RK (RKCK54)</t>
+  </si>
+  <si>
+    <t>LSODA</t>
+  </si>
+  <si>
+    <t>Ref</t>
+  </si>
+  <si>
+    <t>ODEPACK (http://www.netlib.org/odepack/); DASPK (http://www.netlib.org/ode/) (in FORTRAN)</t>
+  </si>
+  <si>
+    <t>LIBLSODA (https://github.com/sdwfrost/liblsoda) + ported and original algorithms  (in C)</t>
+  </si>
+  <si>
+    <t>DLSODA (http://www.netlib.org/odepack/) (translated to C++)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black box solver, cannot change method or solver parameters </t>
+  </si>
+  <si>
+    <t>Boost::odeint (https://github.com/boostorg/odeint) (C++)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,6 +227,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -231,13 +245,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -251,10 +265,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -263,18 +278,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -553,25 +572,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="25.77734375" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.88671875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="14.21875" style="3" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="17.21875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" style="3" customWidth="1"/>
-    <col min="9" max="10" width="9.33203125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="10.77734375" style="3" customWidth="1"/>
-    <col min="12" max="12" width="81.44140625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="17" style="5" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="5"/>
+    <col min="2" max="3" width="25.77734375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="14.21875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17.21875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="16.44140625" style="3" customWidth="1"/>
+    <col min="10" max="11" width="9.33203125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="10.77734375" style="3" customWidth="1"/>
+    <col min="13" max="13" width="81.44140625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="17" style="5" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="2" customFormat="1" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,252 +598,258 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>39</v>
+        <v>17</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="8"/>
+      <c r="D2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="I2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="102.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="E5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="L2" s="3" t="s">
+      <c r="E6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="E7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="102.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3" t="s">
+      <c r="I8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="28.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="L7" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="M7" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>54</v>
+      <c r="N8" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>